<commit_message>
Daily slate 2026-06-15 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-13.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-13.xlsx
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="E4" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F4" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="G4" t="n">
-        <v>52.8</v>
+        <v>51.6</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E5" t="n">
         <v>45</v>
       </c>
       <c r="F5" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G5" t="n">
-        <v>52.9</v>
+        <v>51.7</v>
       </c>
     </row>
     <row r="6">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E7" t="n">
         <v>65</v>
       </c>
       <c r="F7" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G7" t="n">
-        <v>48.9</v>
+        <v>48.1</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>211</v>
+        <v>236</v>
       </c>
       <c r="E8" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F8" t="n">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="G8" t="n">
-        <v>46</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E9" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F9" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>55.2</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1230</v>
+        <v>1295</v>
       </c>
       <c r="E11" t="n">
-        <v>752</v>
+        <v>785</v>
       </c>
       <c r="F11" t="n">
-        <v>478</v>
+        <v>510</v>
       </c>
       <c r="G11" t="n">
-        <v>61.1</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="E12" t="n">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="F12" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G12" t="n">
-        <v>68.2</v>
+        <v>68.40000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E13" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F13" t="n">
         <v>68</v>
       </c>
       <c r="G13" t="n">
-        <v>55.6</v>
+        <v>55.8</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>370</v>
+        <v>387</v>
       </c>
       <c r="E14" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="F14" t="n">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="G14" t="n">
-        <v>31.6</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>511</v>
+        <v>523</v>
       </c>
       <c r="E15" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F15" t="n">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="G15" t="n">
-        <v>23.1</v>
+        <v>23.3</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E16" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F16" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G16" t="n">
-        <v>25.8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4740</v>
+        <v>5004</v>
       </c>
       <c r="E17" t="n">
-        <v>958</v>
+        <v>1017</v>
       </c>
       <c r="F17" t="n">
-        <v>3782</v>
+        <v>3987</v>
       </c>
       <c r="G17" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
     </row>
   </sheetData>
@@ -1351,10 +1351,10 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>30.8</v>
+        <v>21.1</v>
       </c>
       <c r="Y4" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="Z4" t="n">
         <v>65.7</v>
@@ -1579,46 +1579,46 @@
         <v>348</v>
       </c>
       <c r="D7" t="n">
-        <v>61.1</v>
+        <v>60.6</v>
       </c>
       <c r="E7" t="n">
-        <v>1230</v>
+        <v>1295</v>
       </c>
       <c r="F7" t="n">
-        <v>68.2</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="H7" t="n">
-        <v>55.6</v>
+        <v>55.8</v>
       </c>
       <c r="I7" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J7" t="n">
-        <v>31.6</v>
+        <v>31.3</v>
       </c>
       <c r="K7" t="n">
-        <v>370</v>
+        <v>387</v>
       </c>
       <c r="L7" t="n">
-        <v>23.1</v>
+        <v>23.3</v>
       </c>
       <c r="M7" t="n">
-        <v>511</v>
+        <v>523</v>
       </c>
       <c r="N7" t="n">
-        <v>25.8</v>
+        <v>26</v>
       </c>
       <c r="O7" t="n">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="P7" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>4740</v>
+        <v>5004</v>
       </c>
       <c r="R7" t="n">
         <v>57.2</v>
@@ -1627,10 +1627,10 @@
         <v>388</v>
       </c>
       <c r="T7" t="n">
-        <v>52.8</v>
+        <v>51.6</v>
       </c>
       <c r="U7" t="n">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
@@ -1639,10 +1639,10 @@
         <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>46</v>
+        <v>42.8</v>
       </c>
       <c r="Y7" t="n">
-        <v>211</v>
+        <v>236</v>
       </c>
       <c r="Z7" t="n">
         <v>51.5</v>
@@ -1651,22 +1651,22 @@
         <v>134</v>
       </c>
       <c r="AB7" t="n">
-        <v>52.9</v>
+        <v>51.7</v>
       </c>
       <c r="AC7" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AD7" t="n">
-        <v>48.9</v>
+        <v>48.1</v>
       </c>
       <c r="AE7" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="AF7" t="n">
-        <v>55.2</v>
+        <v>55</v>
       </c>
       <c r="AG7" t="n">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>